<commit_message>
checkpoint corrected offline audit 20260814-live-003
</commit_message>
<xml_diff>
--- a/output/20260814-live-003-线下活动核销结果.xlsx
+++ b/output/20260814-live-003-线下活动核销结果.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'堆头-逐店核验'!$A$3:$N$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'堆头-销售检查'!$A$12:$H$49</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'堆头-照片文件检查'!$A$3:$I$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'堆头-异常补证'!$A$3:$F$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'堆头-异常补证'!$A$3:$F$12</definedName>
   </definedNames>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
@@ -97,7 +97,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -122,6 +122,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -157,7 +162,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -181,9 +186,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -194,6 +196,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -717,19 +725,19 @@
         <f>C5-E5</f>
         <v/>
       </c>
-      <c r="G5" s="9" t="inlineStr">
-        <is>
-          <t>human_review</t>
+      <c r="G5" s="7" t="inlineStr">
+        <is>
+          <t>partial_pass</t>
         </is>
       </c>
       <c r="H5" s="4" t="inlineStr">
         <is>
-          <t>0/20家通过；20家补证</t>
+          <t>14/20家通过；6家补证</t>
         </is>
       </c>
       <c r="I5" s="4" t="inlineStr">
         <is>
-          <t>合同第1家“66广场家家欣”未通过：照片缺失、门店未匹配。；合同第2家“百佳华松岗店”未通过：照片缺失。；合同第3家“百佳华百货（公明店）”未通过：照片缺失。</t>
+          <t>合同第1家“66广场家家欣”未通过：门店未匹配。；合同第6家“金大福（东浦金正和总店）”未通过：期间未通过、门店未匹配、陈列标准未通过。；合同第10家“挺拇指生活超市（横沥店）”未通过：门店未匹配。</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
@@ -739,35 +747,35 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B6" s="10" t="n"/>
-      <c r="C6" s="10">
+      <c r="B6" s="9" t="n"/>
+      <c r="C6" s="9">
         <f>SUM(C4:C5)</f>
         <v/>
       </c>
-      <c r="D6" s="10">
+      <c r="D6" s="9">
         <f>SUM(D4:D5)</f>
         <v/>
       </c>
-      <c r="E6" s="10">
+      <c r="E6" s="9">
         <f>SUM(E4:E5)</f>
         <v/>
       </c>
-      <c r="F6" s="10">
+      <c r="F6" s="9">
         <f>SUM(F4:F5)</f>
         <v/>
       </c>
-      <c r="G6" s="10">
+      <c r="G6" s="9">
         <f>IF(F6=0,"全部通过","存在暂挂/补证")</f>
         <v/>
       </c>
-      <c r="H6" s="10" t="n"/>
-      <c r="I6" s="10" t="n"/>
-      <c r="J6" s="10" t="n"/>
+      <c r="H6" s="9" t="n"/>
+      <c r="I6" s="9" t="n"/>
+      <c r="J6" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:J6"/>
@@ -789,7 +797,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -847,719 +855,285 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="9" t="n">
+      <c r="A4" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B4" s="9" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D4" s="9" t="inlineStr">
-        <is>
-          <t>合同第1家“66广场家家欣”未通过：照片缺失、门店未匹配。
+      <c r="D4" s="14" t="inlineStr">
+        <is>
+          <t>合同第1家“66广场家家欣”未通过：门店未匹配。
 来源：核销资料-诚成26年4月【堆头20家】/堆头照片/1.厚街汉邦66广场家家欣.jpg</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="E4" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F4" s="9" t="inlineStr">
-        <is>
-          <t>补充“66广场家家欣”与“厚街镇汉邦广场”的地址/入驻关系证明，或提供同日带完整门店名称与地点水印的现场照片。；补齐缺失原始照片文件</t>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>补充“66广场家家欣”与“厚街镇汉邦广场”的地址/入驻关系证明，或提供同日带完整门店名称与地点水印的现场照片。</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="n">
+      <c r="A5" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
-        <is>
-          <t>合同第2家“百佳华松岗店”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/2.松岗百佳华.jpg</t>
-        </is>
-      </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="D5" s="14" t="inlineStr">
+        <is>
+          <t>合同第6家“金大福（东浦金正和总店）”未通过：期间未通过、门店未匹配、陈列标准未通过。
+来源：核销资料-诚成26年4月【堆头20家】/堆头照片/6.东浦金正和.jpg</t>
+        </is>
+      </c>
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
-        <is>
-          <t>如需严格同店证明，补充“百佳华松岗店”与“百佳华超市(松岗百佳华商场店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>补充活动期内带可见日期、完整门店名称/地点水印的现场全景原图。；补充能清楚证明1平方米占地或至少4纵陈列的宽角度照片/尺寸标识。</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9" t="n">
+      <c r="A6" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>合同第3家“百佳华百货（公明店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/3.公明百佳华.jpg</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="D6" s="14" t="inlineStr">
+        <is>
+          <t>合同第10家“挺拇指生活超市（横沥店）”未通过：门店未匹配。
+来源：核销资料-诚成26年4月【堆头20家】/堆头照片/10-1挺拇指生活超市(横沥店).jpg、核销资料-诚成26年4月【堆头20家】/堆头照片/10-2挺拇指生活超市(横沥店).jpg</t>
+        </is>
+      </c>
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F6" s="9" t="inlineStr">
-        <is>
-          <t>补充公明店更名、门店编码或地址一致性证明。；补齐缺失原始照片文件</t>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>补充“挺拇指生活超市(横沥店)”位于或更名自“南铭购物乐园”的正式地址/门店映射，或提供带合同门店名称水印的现场照片。</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9" t="n">
+      <c r="A7" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C7" s="9" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>合同第4家“百佳华佳漾汇（新桥店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/4.新桥百佳华.jpg</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="D7" s="14" t="inlineStr">
+        <is>
+          <t>合同第11家“人人购物广场荟和二店”未通过：门店未匹配。
+来源：核销资料-诚成26年4月【堆头20家】/堆头照片/11.人人购物荟和超市.jpg</t>
+        </is>
+      </c>
+      <c r="E7" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>补充“荟和二店”与“人人购物同乐店”的门店编码、地址或更名证明，或提供合同门店对应照片。</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9" t="n">
+      <c r="A8" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>合同第5家“华都超市（东坑大道北店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/5.华都超市(东坑大道北店).jpg</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="D8" s="14" t="inlineStr">
+        <is>
+          <t>合同第14家“润家连锁超市（美联购物中心店）”未通过：门店未匹配。
+来源：核销资料-诚成26年4月【堆头20家】/堆头照片/14.润家连锁超市(美联购物中心店).jpg</t>
+        </is>
+      </c>
+      <c r="E8" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F8" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>提供“深圳紫云快捷宾馆”定位与润家连锁超市(美联购物中心店)同址的权威地址证明，或重拍带合同门店地点水印的现场照片。</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9" t="n">
+      <c r="A9" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>high</t>
         </is>
       </c>
-      <c r="C9" s="9" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
         </is>
       </c>
-      <c r="D9" s="9" t="inlineStr">
-        <is>
-          <t>合同第6家“金大福（东浦金正和总店）”未通过：照片缺失、期间未通过、门店未匹配、陈列标准未通过。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/6.东浦金正和.jpg</t>
-        </is>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="D9" s="14" t="inlineStr">
+        <is>
+          <t>合同第15家“百佳华（石岩店）”未通过：门店未匹配。
+来源：核销资料-诚成26年4月【堆头20家】/堆头照片/15。石岩百佳华.jpg</t>
+        </is>
+      </c>
+      <c r="E9" s="14" t="inlineStr">
         <is>
           <t>暂不支持该店1000.00元费用。</t>
         </is>
       </c>
-      <c r="F9" s="9" t="inlineStr">
-        <is>
-          <t>补充活动期内带可见日期、完整门店名称/地点水印的现场全景原图。；补充能清楚证明1平方米占地或至少4纵陈列的宽角度照片/尺寸标识。；补齐缺失原始照片文件</t>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>补充百佳华(石岩店)与“佳华豪苑”的权威地址/入驻关系证明，或提供带完整门店名地点水印的清晰原图。</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="n">
+      <c r="A10" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>合同第7家“古原千禧（U·ONE 优城店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/7.宝安优城店.jpg</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>如需严格名称一致，补充U·ONE优城店与水印“古原千禧(优城店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>PHOTO_ORIGINAL_METADATA_ABSENT</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>照片缺少可用的EXIF拍摄时间或GPS，主要依赖画面水印。</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="inlineStr">
+        <is>
+          <t>无法从原始文件元数据独立验证拍摄时空。</t>
+        </is>
+      </c>
+      <c r="F10" s="7" t="inlineStr">
+        <is>
+          <t>保留原始拍摄文件，或补充平台定位/签到记录。</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9" t="n">
+      <c r="A11" s="7" t="n">
         <v>8</v>
       </c>
-      <c r="B11" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C11" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D11" s="9" t="inlineStr">
-        <is>
-          <t>合同第8家“虎门家家欣”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/8.虎门赤岗家家欣.jpg</t>
-        </is>
-      </c>
-      <c r="E11" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F11" s="9" t="inlineStr">
-        <is>
-          <t>补充“虎门家家欣”与“赤岗家家欣商场”的地址、门店编码或组织关系证明。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="9" t="n">
-        <v>9</v>
-      </c>
-      <c r="B12" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>合同第9家“花都宜多”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/9.花都宜多.jpg</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F12" s="9" t="inlineStr">
-        <is>
-          <t>补充“花都宜多”与“炭步宜多百货”的门店编码或地址映射。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="9" t="n">
-        <v>10</v>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D13" s="9" t="inlineStr">
-        <is>
-          <t>合同第10家“挺拇指生活超市（横沥店）”未通过：照片缺失、门店未匹配。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/10-1挺拇指生活超市(横沥店).jpg、核销资料-诚成26年4月【堆头20家】/堆头照片/10-2挺拇指生活超市(横沥店).jpg</t>
-        </is>
-      </c>
-      <c r="E13" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F13" s="9" t="inlineStr">
-        <is>
-          <t>补充“挺拇指生活超市(横沥店)”位于或更名自“南铭购物乐园”的正式地址/门店映射，或提供带合同门店名称水印的现场照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="n">
-        <v>11</v>
-      </c>
-      <c r="B14" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>合同第11家“人人购物广场荟和二店”未通过：照片缺失、门店未匹配。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/11.人人购物荟和超市.jpg</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F14" s="9" t="inlineStr">
-        <is>
-          <t>补充“荟和二店”与“人人购物同乐店”的门店编码、地址或更名证明，或提供合同门店对应照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="B15" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D15" s="9" t="inlineStr">
-        <is>
-          <t>合同第12家“三乐购物广场（森扬商业广场店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/12.三乐购物广场(森扬商业广场店).jpg</t>
-        </is>
-      </c>
-      <c r="E15" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F15" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="9" t="n">
-        <v>13</v>
-      </c>
-      <c r="B16" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>合同第13家“沙井九龙”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/13.沙井九龙.jpg</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F16" s="9" t="inlineStr">
-        <is>
-          <t>如需严格名称一致，补充“沙井九龙”与“九龙购物中心(宝安沙井店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="9" t="n">
-        <v>14</v>
-      </c>
-      <c r="B17" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D17" s="9" t="inlineStr">
-        <is>
-          <t>合同第14家“润家连锁超市（美联购物中心店）”未通过：照片缺失、门店未匹配。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/14.润家连锁超市(美联购物中心店).jpg</t>
-        </is>
-      </c>
-      <c r="E17" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F17" s="9" t="inlineStr">
-        <is>
-          <t>提供“深圳紫云快捷宾馆”定位与润家连锁超市(美联购物中心店)同址的权威地址证明，或重拍带合同门店地点水印的现场照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="9" t="n">
-        <v>15</v>
-      </c>
-      <c r="B18" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>合同第15家“百佳华（石岩店）”未通过：照片缺失、门店未匹配。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/15。石岩百佳华.jpg</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="inlineStr">
-        <is>
-          <t>补充百佳华(石岩店)与“佳华豪苑”的权威地址/入驻关系证明，或提供带完整门店名地点水印的清晰原图。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="n">
-        <v>16</v>
-      </c>
-      <c r="B19" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C19" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D19" s="9" t="inlineStr">
-        <is>
-          <t>合同第16家“田心金正和”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/16.田心金正和.jpg</t>
-        </is>
-      </c>
-      <c r="E19" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="9" t="n">
-        <v>17</v>
-      </c>
-      <c r="B20" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
-        <is>
-          <t>合同第17家“荟和超市（莹展荟店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/17·荟和超市(莹展荟店).jpg</t>
-        </is>
-      </c>
-      <c r="E20" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F20" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="9" t="n">
-        <v>18</v>
-      </c>
-      <c r="B21" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C21" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D21" s="9" t="inlineStr">
-        <is>
-          <t>合同第18家“三乐购物广场（坦洲店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/18.三乐购物广场(坦洲店).jpg</t>
-        </is>
-      </c>
-      <c r="E21" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F21" s="9" t="inlineStr">
-        <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="9" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>合同第19家“大康惠福源商业广场”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/19.福源大康惠.jpg</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F22" s="9" t="inlineStr">
-        <is>
-          <t>补充“大康惠福源商业广场”与“福源商业广场”的门店/地址映射。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="9" t="n">
-        <v>20</v>
-      </c>
-      <c r="B23" s="9" t="inlineStr">
-        <is>
-          <t>high</t>
-        </is>
-      </c>
-      <c r="C23" s="9" t="inlineStr">
-        <is>
-          <t>STORE_DISPLAY_EVIDENCE_INCOMPLETE</t>
-        </is>
-      </c>
-      <c r="D23" s="9" t="inlineStr">
-        <is>
-          <t>合同第20家“好多宝精选超市（龙眼市场店）”未通过：照片缺失。
-来源：核销资料-诚成26年4月【堆头20家】/堆头照片/20.好多宝精选超市(龙眼市场店).jpg</t>
-        </is>
-      </c>
-      <c r="E23" s="9" t="inlineStr">
-        <is>
-          <t>暂不支持该店1000.00元费用。</t>
-        </is>
-      </c>
-      <c r="F23" s="9" t="inlineStr">
-        <is>
-          <t>补充好多宝精选超市(龙眼市场店)在“龙眼市场(龙眼路)”的门店编码、地址或入驻证明。；补齐缺失原始照片文件</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="7" t="n">
-        <v>21</v>
-      </c>
-      <c r="B24" s="7" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C24" s="7" t="inlineStr">
-        <is>
-          <t>PHOTO_ORIGINAL_METADATA_ABSENT</t>
-        </is>
-      </c>
-      <c r="D24" s="7" t="inlineStr">
-        <is>
-          <t>照片缺少可用的EXIF拍摄时间或GPS，主要依赖画面水印。</t>
-        </is>
-      </c>
-      <c r="E24" s="7" t="inlineStr">
-        <is>
-          <t>无法从原始文件元数据独立验证拍摄时空。</t>
-        </is>
-      </c>
-      <c r="F24" s="7" t="inlineStr">
-        <is>
-          <t>保留原始拍摄文件，或补充平台定位/签到记录。</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="7" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>medium</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>SALES_DATA_NOT_STORE_LEVEL</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>销售Excel为经销商汇总，不能拆分到合同中的各门店。
 来源：C:\Users\EDY\Desktop\新建文件夹\offline-activity-audit\input\.prepared\20260814-live-003\sources\promotional_display\核销资料-诚成26年4月【堆头20家】\2026年4月销售明细20260509164207765.xlsx</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>销售数据只能证明活动期总体销售，不能独立证明逐店执行。</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>如政策要求逐店销售佐证，补交门店级POS或出库明细。</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="7" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="7" t="n">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C26" s="7" t="inlineStr">
+      <c r="C12" s="7" t="inlineStr">
         <is>
           <t>SALES_EXCEL_EXTERNAL_LINKS</t>
         </is>
       </c>
-      <c r="D26" s="7" t="inlineStr">
+      <c r="D12" s="7" t="inlineStr">
         <is>
           <t>销售Excel有36个公式引用缺失的外部工作簿。
 来源：H10,H11,H16,H17,H21,H22,H27,H30,H31,H33,H34,H9,L11,L13,L14,L15,L16,L17,L2,L20</t>
         </is>
       </c>
-      <c r="E26" s="7" t="inlineStr">
+      <c r="E12" s="7" t="inlineStr">
         <is>
           <t>部分单位或零售价无法在当前文件内独立重算。</t>
         </is>
       </c>
-      <c r="F26" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>补交被引用主数据或将外链转为可追溯静态值。</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F26"/>
+  <autoFilter ref="A3:F12"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -2444,58 +2018,58 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10">
+      <c r="B14" s="9" t="n"/>
+      <c r="C14" s="9" t="n"/>
+      <c r="D14" s="9" t="n"/>
+      <c r="E14" s="9" t="n"/>
+      <c r="F14" s="9">
         <f>SUM(F4:F13)</f>
         <v/>
       </c>
-      <c r="G14" s="10">
+      <c r="G14" s="9">
         <f>SUM(G4:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="10">
+      <c r="H14" s="9">
         <f>SUM(H4:H13)</f>
         <v/>
       </c>
-      <c r="I14" s="10" t="n"/>
-      <c r="J14" s="10">
+      <c r="I14" s="9" t="n"/>
+      <c r="J14" s="9">
         <f>SUM(J4:J13)</f>
         <v/>
       </c>
-      <c r="K14" s="10">
+      <c r="K14" s="9">
         <f>SUM(K4:K13)</f>
         <v/>
       </c>
-      <c r="L14" s="10">
+      <c r="L14" s="9">
         <f>SUM(L4:L13)</f>
         <v/>
       </c>
-      <c r="M14" s="10">
+      <c r="M14" s="9">
         <f>SUM(M4:M13)</f>
         <v/>
       </c>
-      <c r="N14" s="10">
+      <c r="N14" s="9">
         <f>SUM(N4:N13)</f>
         <v/>
       </c>
-      <c r="O14" s="10" t="n"/>
-      <c r="P14" s="10">
+      <c r="O14" s="9" t="n"/>
+      <c r="P14" s="9">
         <f>SUM(P4:P13)</f>
         <v/>
       </c>
-      <c r="Q14" s="10">
+      <c r="Q14" s="9">
         <f>SUM(Q4:Q13)</f>
         <v/>
       </c>
-      <c r="R14" s="10" t="n"/>
+      <c r="R14" s="9" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:R14"/>
@@ -5821,24 +5395,24 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="12" t="inlineStr">
+      <c r="A74" s="11" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B74" s="12" t="n"/>
-      <c r="C74" s="12" t="n"/>
-      <c r="D74" s="12" t="n"/>
-      <c r="E74" s="12" t="n"/>
-      <c r="F74" s="13">
+      <c r="B74" s="11" t="n"/>
+      <c r="C74" s="11" t="n"/>
+      <c r="D74" s="11" t="n"/>
+      <c r="E74" s="11" t="n"/>
+      <c r="F74" s="12">
         <f>SUM(F4:F73)</f>
         <v/>
       </c>
-      <c r="G74" s="12" t="n"/>
-      <c r="H74" s="12" t="n"/>
-      <c r="I74" s="12" t="n"/>
-      <c r="J74" s="12" t="n"/>
-      <c r="K74" s="13">
+      <c r="G74" s="11" t="n"/>
+      <c r="H74" s="11" t="n"/>
+      <c r="I74" s="11" t="n"/>
+      <c r="J74" s="11" t="n"/>
+      <c r="K74" s="12">
         <f>SUM(K4:K73)</f>
         <v/>
       </c>
@@ -6215,31 +5789,31 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="12">
         <f>SUM(B4:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="12">
         <f>SUM(C4:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="12" t="n"/>
-      <c r="E11" s="13">
+      <c r="D11" s="11" t="n"/>
+      <c r="E11" s="12">
         <f>SUM(E4:E10)</f>
         <v/>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="12">
         <f>SUM(F4:F10)</f>
         <v/>
       </c>
-      <c r="G11" s="12" t="n"/>
-      <c r="H11" s="12" t="n"/>
-      <c r="I11" s="12" t="n"/>
+      <c r="G11" s="11" t="n"/>
+      <c r="H11" s="11" t="n"/>
+      <c r="I11" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:I11"/>
@@ -7087,12 +6661,12 @@
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>画面显示参半礼盒/牙膏在大型多层岛柜上多列陈列，可见至少4纵陈列特征。；水印地点与合同门店名称未形成独立一致映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=2bc5b681403c0d0e05ba6394449fd73b18e211370dbdfc3b1e3166678fb33aad，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/1.厚街汉邦66广场家家欣.jpg</t>
+          <t>画面显示参半礼盒/牙膏在大型多层岛柜上多列陈列，可见至少4纵陈列特征。；水印地点与合同门店名称未形成独立一致映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=2bc5b681403c0d0e05ba6394449fd73b18e211370dbdfc3b1e3166678fb33aad，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N4" s="4" t="inlineStr">
         <is>
-          <t>补充“66广场家家欣”与“厚街镇汉邦广场”的地址/入驻关系证明，或提供同日带完整门店名称与地点水印的现场照片。；补齐缺失原始照片文件</t>
+          <t>补充“66广场家家欣”与“厚街镇汉邦广场”的地址/入驻关系证明，或提供同日带完整门店名称与地点水印的现场照片。</t>
         </is>
       </c>
     </row>
@@ -7143,9 +6717,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K5" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L5" s="6">
@@ -7154,12 +6728,12 @@
       </c>
       <c r="M5" s="4" t="inlineStr">
         <is>
-          <t>参半产品在多层货架上形成多列陈列，可见至少4纵陈列特征。；合同简称与水印全称并非逐字相同。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=12b86e89b2996c4ee22ce55cfa65249237f10c2651963f0a74d6748f6fbdf29f，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/2.松岗百佳华.jpg</t>
+          <t>参半产品在多层货架上形成多列陈列，可见至少4纵陈列特征。；合同简称与水印全称并非逐字相同。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=12b86e89b2996c4ee22ce55cfa65249237f10c2651963f0a74d6748f6fbdf29f，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N5" s="4" t="inlineStr">
         <is>
-          <t>如需严格同店证明，补充“百佳华松岗店”与“百佳华超市(松岗百佳华商场店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+          <t>如需严格同店证明，补充“百佳华松岗店”与“百佳华超市(松岗百佳华商场店)”的门店编码或地址映射。</t>
         </is>
       </c>
     </row>
@@ -7210,9 +6784,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K6" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K6" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L6" s="6">
@@ -7221,12 +6795,12 @@
       </c>
       <c r="M6" s="4" t="inlineStr">
         <is>
-          <t>多层端架上可见参半礼盒多列陈列，至少4个纵向陈列位可辨。；“百佳华百货”与“百佳华佳漾汇”的名称变化未附正式说明。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=334f7fe95b8f70a59cf89c0e2b65a47ba1a19c70d8b1695a51ecd59bdce07463，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/3.公明百佳华.jpg</t>
+          <t>多层端架上可见参半礼盒多列陈列，至少4个纵向陈列位可辨。；“百佳华百货”与“百佳华佳漾汇”的名称变化未附正式说明。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=334f7fe95b8f70a59cf89c0e2b65a47ba1a19c70d8b1695a51ecd59bdce07463，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N6" s="4" t="inlineStr">
         <is>
-          <t>补充公明店更名、门店编码或地址一致性证明。；补齐缺失原始照片文件</t>
+          <t>补充公明店更名、门店编码或地址一致性证明。</t>
         </is>
       </c>
     </row>
@@ -7277,9 +6851,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K7" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L7" s="6">
@@ -7288,12 +6862,12 @@
       </c>
       <c r="M7" s="4" t="inlineStr">
         <is>
-          <t>画面可见多层端架及参半礼盒/盒装产品多列陈列，满足至少4纵陈列的可见特征。；原图仅600×800，细节分辨率有限。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=df7c36d02303fc3b8df13e63888d0dcfed56860ca91d2a86501f67168d32c3ff，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/4.新桥百佳华.jpg</t>
+          <t>画面可见多层端架及参半礼盒/盒装产品多列陈列，满足至少4纵陈列的可见特征。；原图仅600×800，细节分辨率有限。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=df7c36d02303fc3b8df13e63888d0dcfed56860ca91d2a86501f67168d32c3ff，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N7" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -7344,9 +6918,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K8" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L8" s="6">
@@ -7355,12 +6929,12 @@
       </c>
       <c r="M8" s="4" t="inlineStr">
         <is>
-          <t>画面可见参半产品在多层岛柜上成组、多列陈列，至少4纵陈列特征清晰。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=61e7f18669fe68e0686638d9bf53e6e488e8ce9ccb78192cdb6647915337dad0，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/5.华都超市(东坑大道北店).jpg</t>
+          <t>画面可见参半产品在多层岛柜上成组、多列陈列，至少4纵陈列特征清晰。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=61e7f18669fe68e0686638d9bf53e6e488e8ce9ccb78192cdb6647915337dad0，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N8" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -7414,12 +6988,12 @@
       </c>
       <c r="M9" s="4" t="inlineStr">
         <is>
-          <t>画面可见参半3+2礼盒及竖盒放在红色促销台上，但单一正面角度无法可靠确认1平方米占地，且4纵陈列计数不够明确。；缺少任何画面内日期和门店/地点水印。；JPEG文件EXIF为空，无法从元数据独立验证拍摄日期或地点。；文件SHA-256=5443f87d47fe6646e5da357f0e53a41c8934f58255619fe749eae9b7ad9596a0，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/6.东浦金正和.jpg</t>
+          <t>画面可见参半3+2礼盒及竖盒放在红色促销台上，但单一正面角度无法可靠确认1平方米占地，且4纵陈列计数不够明确。；缺少任何画面内日期和门店/地点水印。；JPEG文件EXIF为空，无法从元数据独立验证拍摄日期或地点。；文件SHA-256=5443f87d47fe6646e5da357f0e53a41c8934f58255619fe749eae9b7ad9596a0，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N9" s="4" t="inlineStr">
         <is>
-          <t>补充活动期内带可见日期、完整门店名称/地点水印的现场全景原图。；补充能清楚证明1平方米占地或至少4纵陈列的宽角度照片/尺寸标识。；补齐缺失原始照片文件</t>
+          <t>补充活动期内带可见日期、完整门店名称/地点水印的现场全景原图。；补充能清楚证明1平方米占地或至少4纵陈列的宽角度照片/尺寸标识。</t>
         </is>
       </c>
     </row>
@@ -7470,9 +7044,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K10" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K10" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L10" s="6">
@@ -7481,12 +7055,12 @@
       </c>
       <c r="M10" s="4" t="inlineStr">
         <is>
-          <t>多层端架上参半礼盒/盒装产品有多列、多层陈列，可见至少4纵陈列特征。；水印省略合同中的“U·ONE”。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=80ff9c92a5eb1b780e9b0002a5d99c5239d71f592406992133c1e49e77e5834f，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/7.宝安优城店.jpg</t>
+          <t>多层端架上参半礼盒/盒装产品有多列、多层陈列，可见至少4纵陈列特征。；水印省略合同中的“U·ONE”。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=80ff9c92a5eb1b780e9b0002a5d99c5239d71f592406992133c1e49e77e5834f，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N10" s="4" t="inlineStr">
         <is>
-          <t>如需严格名称一致，补充U·ONE优城店与水印“古原千禧(优城店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+          <t>如需严格名称一致，补充U·ONE优城店与水印“古原千禧(优城店)”的门店编码或地址映射。</t>
         </is>
       </c>
     </row>
@@ -7537,9 +7111,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K11" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K11" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L11" s="6">
@@ -7548,12 +7122,12 @@
       </c>
       <c r="M11" s="4" t="inlineStr">
         <is>
-          <t>多层端架上参半礼盒至少形成4个纵向陈列位。；原图仅600×800，且未提供赤岗与合同“虎门”分店的地址关系。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a397af48c29cc108f54a66ac21d7aec414e79f20838ee3bb2e4851619d1f9e0a，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/8.虎门赤岗家家欣.jpg</t>
+          <t>多层端架上参半礼盒至少形成4个纵向陈列位。；原图仅600×800，且未提供赤岗与合同“虎门”分店的地址关系。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a397af48c29cc108f54a66ac21d7aec414e79f20838ee3bb2e4851619d1f9e0a，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N11" s="4" t="inlineStr">
         <is>
-          <t>补充“虎门家家欣”与“赤岗家家欣商场”的地址、门店编码或组织关系证明。；补齐缺失原始照片文件</t>
+          <t>补充“虎门家家欣”与“赤岗家家欣商场”的地址、门店编码或组织关系证明。</t>
         </is>
       </c>
     </row>
@@ -7604,9 +7178,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K12" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K12" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L12" s="6">
@@ -7615,12 +7189,12 @@
       </c>
       <c r="M12" s="4" t="inlineStr">
         <is>
-          <t>画面为大型多面岛柜，参半牙膏、礼盒等产品多层多列陈列，可见面积/纵列明显超过最低特征。；合同简称未列“炭步”，未附门店编码。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=37a3bb4647855bff6147f370f02897142fb739c3b1f015546c9701327ca79c87，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/9.花都宜多.jpg</t>
+          <t>画面为大型多面岛柜，参半牙膏、礼盒等产品多层多列陈列，可见面积/纵列明显超过最低特征。；合同简称未列“炭步”，未附门店编码。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=37a3bb4647855bff6147f370f02897142fb739c3b1f015546c9701327ca79c87，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N12" s="4" t="inlineStr">
         <is>
-          <t>补充“花都宜多”与“炭步宜多百货”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+          <t>补充“花都宜多”与“炭步宜多百货”的门店编码或地址映射。</t>
         </is>
       </c>
     </row>
@@ -7682,12 +7256,12 @@
       </c>
       <c r="M13" s="4" t="inlineStr">
         <is>
-          <t>10-1为多层端架全景，10-2为另一侧近景；合并观察可见参半产品多层多列陈列，至少4纵陈列特征明确。；可见地点名称与合同门店名称不同，未提供商场入驻/更名映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；10-1挺拇指生活超市(横沥店).jpg SHA-256=f12dd735b31b0e3be209767b443a5dde76af047139821839e1c380befa2f17ba、精确哈希出现次数1；10-2挺拇指生活超市(横沥店).jpg SHA-256=1d4f8b92c71131ea2dbe09e06cff7496a82afca0ba4d7fced7ab272948670884、精确哈希出现次数1；两图内容不同，感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/10-1挺拇指生活超市(横沥店).jpg、核销资料-诚成26年4月【堆头20家】/堆头照片/10-2挺拇指生活超市(横沥店).jpg</t>
+          <t>10-1为多层端架全景，10-2为另一侧近景；合并观察可见参半产品多层多列陈列，至少4纵陈列特征明确。；可见地点名称与合同门店名称不同，未提供商场入驻/更名映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；10-1挺拇指生活超市(横沥店).jpg SHA-256=f12dd735b31b0e3be209767b443a5dde76af047139821839e1c380befa2f17ba、精确哈希出现次数1；10-2挺拇指生活超市(横沥店).jpg SHA-256=1d4f8b92c71131ea2dbe09e06cff7496a82afca0ba4d7fced7ab272948670884、精确哈希出现次数1；两图内容不同，感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N13" s="4" t="inlineStr">
         <is>
-          <t>补充“挺拇指生活超市(横沥店)”位于或更名自“南铭购物乐园”的正式地址/门店映射，或提供带合同门店名称水印的现场照片。；补齐缺失原始照片文件</t>
+          <t>补充“挺拇指生活超市(横沥店)”位于或更名自“南铭购物乐园”的正式地址/门店映射，或提供带合同门店名称水印的现场照片。</t>
         </is>
       </c>
     </row>
@@ -7749,12 +7323,12 @@
       </c>
       <c r="M14" s="4" t="inlineStr">
         <is>
-          <t>大型多层端架上参半产品有多列多层陈列，至少4纵陈列特征明确。；水印指向“同乐店”，合同指向“二店”。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=7cf34a44ba05a348179771b0c36be20c19f6a0a76fb0c72fc6742c1070011f87，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/11.人人购物荟和超市.jpg</t>
+          <t>大型多层端架上参半产品有多列多层陈列，至少4纵陈列特征明确。；水印指向“同乐店”，合同指向“二店”。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=7cf34a44ba05a348179771b0c36be20c19f6a0a76fb0c72fc6742c1070011f87，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N14" s="4" t="inlineStr">
         <is>
-          <t>补充“荟和二店”与“人人购物同乐店”的门店编码、地址或更名证明，或提供合同门店对应照片。；补齐缺失原始照片文件</t>
+          <t>补充“荟和二店”与“人人购物同乐店”的门店编码、地址或更名证明，或提供合同门店对应照片。</t>
         </is>
       </c>
     </row>
@@ -7805,9 +7379,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K15" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K15" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L15" s="6">
@@ -7816,12 +7390,12 @@
       </c>
       <c r="M15" s="4" t="inlineStr">
         <is>
-          <t>参半产品在宽幅多层陈列柜上多列摆放，上方另有堆叠，至少4纵陈列特征明确。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=817e1b01120475a5f72ab39bce2334a3f0c5d2d7c66d02b0d02e648e70bca0e9，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/12.三乐购物广场(森扬商业广场店).jpg</t>
+          <t>参半产品在宽幅多层陈列柜上多列摆放，上方另有堆叠，至少4纵陈列特征明确。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=817e1b01120475a5f72ab39bce2334a3f0c5d2d7c66d02b0d02e648e70bca0e9，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N15" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -7872,9 +7446,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K16" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L16" s="6">
@@ -7883,12 +7457,12 @@
       </c>
       <c r="M16" s="4" t="inlineStr">
         <is>
-          <t>大型岛柜上参半牙膏多层多列陈列，可见面积及纵列均明显达到合同陈列特征。；合同为简称，未列完整购物中心名称。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=bea6157436ef7f0a45babca793b9fc67e06ac2beacd1b9eae36c44097b0e3888，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/13.沙井九龙.jpg</t>
+          <t>大型岛柜上参半牙膏多层多列陈列，可见面积及纵列均明显达到合同陈列特征。；合同为简称，未列完整购物中心名称。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=bea6157436ef7f0a45babca793b9fc67e06ac2beacd1b9eae36c44097b0e3888，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N16" s="4" t="inlineStr">
         <is>
-          <t>如需严格名称一致，补充“沙井九龙”与“九龙购物中心(宝安沙井店)”的门店编码或地址映射。；补齐缺失原始照片文件</t>
+          <t>如需严格名称一致，补充“沙井九龙”与“九龙购物中心(宝安沙井店)”的门店编码或地址映射。</t>
         </is>
       </c>
     </row>
@@ -7950,12 +7524,12 @@
       </c>
       <c r="M17" s="4" t="inlineStr">
         <is>
-          <t>画面中参半礼盒/牙膏在多层货架上形成多列陈列，至少4纵陈列特征明确。；可见地点指向宾馆，与合同门店名称冲突。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=0589b66788746499b68c9813b97ef042c2d1a239cd70be63056d57f4a9587fe5，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/14.润家连锁超市(美联购物中心店).jpg</t>
+          <t>画面中参半礼盒/牙膏在多层货架上形成多列陈列，至少4纵陈列特征明确。；可见地点指向宾馆，与合同门店名称冲突。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=0589b66788746499b68c9813b97ef042c2d1a239cd70be63056d57f4a9587fe5，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N17" s="4" t="inlineStr">
         <is>
-          <t>提供“深圳紫云快捷宾馆”定位与润家连锁超市(美联购物中心店)同址的权威地址证明，或重拍带合同门店地点水印的现场照片。；补齐缺失原始照片文件</t>
+          <t>提供“深圳紫云快捷宾馆”定位与润家连锁超市(美联购物中心店)同址的权威地址证明，或重拍带合同门店地点水印的现场照片。</t>
         </is>
       </c>
     </row>
@@ -8017,12 +7591,12 @@
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>虽画面略模糊，但多层端架上参半礼盒/盒装产品至少4纵陈列仍可辨。；可见地点是“佳华豪苑”，未提供其与百佳华石岩店同址的证据。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=9845f5c8c808e139ae93bf4a163372cf5e54e7aeb39a8dfbfa1d0aa47e5dfca8，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/15。石岩百佳华.jpg</t>
+          <t>虽画面略模糊，但多层端架上参半礼盒/盒装产品至少4纵陈列仍可辨。；可见地点是“佳华豪苑”，未提供其与百佳华石岩店同址的证据。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=9845f5c8c808e139ae93bf4a163372cf5e54e7aeb39a8dfbfa1d0aa47e5dfca8，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N18" s="4" t="inlineStr">
         <is>
-          <t>补充百佳华(石岩店)与“佳华豪苑”的权威地址/入驻关系证明，或提供带完整门店名地点水印的清晰原图。；补齐缺失原始照片文件</t>
+          <t>补充百佳华(石岩店)与“佳华豪苑”的权威地址/入驻关系证明，或提供带完整门店名地点水印的清晰原图。</t>
         </is>
       </c>
     </row>
@@ -8073,9 +7647,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K19" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L19" s="6">
@@ -8084,12 +7658,12 @@
       </c>
       <c r="M19" s="4" t="inlineStr">
         <is>
-          <t>大型多面岛柜上参半礼盒、牙膏等多层多列陈列，可见面积/纵列明显达到合同陈列特征。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=f00f97dc46a52568db5b292f7edb26bedfbc0d6f786e746acea6a56940a7c500，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/16.田心金正和.jpg</t>
+          <t>大型多面岛柜上参半礼盒、牙膏等多层多列陈列，可见面积/纵列明显达到合同陈列特征。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=f00f97dc46a52568db5b292f7edb26bedfbc0d6f786e746acea6a56940a7c500，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N19" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -8140,9 +7714,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K20" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K20" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L20" s="6">
@@ -8151,12 +7725,12 @@
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>大型多面岛柜上参半盒装产品多层多列陈列，可见面积/纵列明显达到合同陈列特征。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=c6a9ac8b3b620adf996334ec432e725c45b4e302c481354caa4959a97c6f1ef1，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/17·荟和超市(莹展荟店).jpg</t>
+          <t>大型多面岛柜上参半盒装产品多层多列陈列，可见面积/纵列明显达到合同陈列特征。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=c6a9ac8b3b620adf996334ec432e725c45b4e302c481354caa4959a97c6f1ef1，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N20" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -8207,9 +7781,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K21" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K21" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L21" s="6">
@@ -8218,12 +7792,12 @@
       </c>
       <c r="M21" s="4" t="inlineStr">
         <is>
-          <t>多层端架上参半礼盒成组陈列，画面下层可见至少4个纵向陈列位。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=61f0c8113bfbfafd9cc02a2ae69881cb8cc456e911c32c78ba618ab3467153fe，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/18.三乐购物广场(坦洲店).jpg</t>
+          <t>多层端架上参半礼盒成组陈列，画面下层可见至少4个纵向陈列位。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=61f0c8113bfbfafd9cc02a2ae69881cb8cc456e911c32c78ba618ab3467153fe，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N21" s="4" t="inlineStr">
         <is>
-          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。；补齐缺失原始照片文件</t>
+          <t>如制度要求原始定位证明，补充含EXIF/GPS的原始未压缩照片。</t>
         </is>
       </c>
     </row>
@@ -8274,9 +7848,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K22" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L22" s="6">
@@ -8285,12 +7859,12 @@
       </c>
       <c r="M22" s="4" t="inlineStr">
         <is>
-          <t>大型四面岛柜上参半牙膏/礼盒多层多列陈列，可见面积与纵列明显达到合同陈列特征。；水印为缩略名称，未附正式门店名称映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a83b7852588f47ff9fc8c43791eab025aa930eb7efa97d4da13cd54024be754c，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/19.福源大康惠.jpg</t>
+          <t>大型四面岛柜上参半牙膏/礼盒多层多列陈列，可见面积与纵列明显达到合同陈列特征。；水印为缩略名称，未附正式门店名称映射。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a83b7852588f47ff9fc8c43791eab025aa930eb7efa97d4da13cd54024be754c，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N22" s="4" t="inlineStr">
         <is>
-          <t>补充“大康惠福源商业广场”与“福源商业广场”的门店/地址映射。；补齐缺失原始照片文件</t>
+          <t>补充“大康惠福源商业广场”与“福源商业广场”的门店/地址映射。</t>
         </is>
       </c>
     </row>
@@ -8341,9 +7915,9 @@
           <t>未发现</t>
         </is>
       </c>
-      <c r="K23" s="7" t="inlineStr">
-        <is>
-          <t>补证</t>
+      <c r="K23" s="13" t="inlineStr">
+        <is>
+          <t>通过</t>
         </is>
       </c>
       <c r="L23" s="6">
@@ -8352,40 +7926,40 @@
       </c>
       <c r="M23" s="4" t="inlineStr">
         <is>
-          <t>多层端架上参半盒装产品至少形成4个纵向陈列位。；水印只证明龙眼市场地点，未直接显示合同门店品牌。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a2bc6e9f7833a6b2dace149843649c6c2a6b5988e04def5a9bc64d4b2b8740fc，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。；结构化核验引用了不存在的照片文件：核销资料-诚成26年4月【堆头20家】/堆头照片/20.好多宝精选超市(龙眼市场店).jpg</t>
+          <t>多层端架上参半盒装产品至少形成4个纵向陈列位。；水印只证明龙眼市场地点，未直接显示合同门店品牌。；JPEG文件EXIF为空；日期和地点只来自画面内可见水印，未由EXIF/GPS独立验证。；文件SHA-256=a2bc6e9f7833a6b2dace149843649c6c2a6b5988e04def5a9bc64d4b2b8740fc，在本案21张照片中精确哈希出现次数为1；感知指纹筛查未见近似重复。</t>
         </is>
       </c>
       <c r="N23" s="4" t="inlineStr">
         <is>
-          <t>补充好多宝精选超市(龙眼市场店)在“龙眼市场(龙眼路)”的门店编码、地址或入驻证明。；补齐缺失原始照片文件</t>
+          <t>补充好多宝精选超市(龙眼市场店)在“龙眼市场(龙眼路)”的门店编码、地址或入驻证明。</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B24" s="12" t="n"/>
-      <c r="C24" s="12" t="n"/>
-      <c r="D24" s="13">
+      <c r="B24" s="11" t="n"/>
+      <c r="C24" s="11" t="n"/>
+      <c r="D24" s="12">
         <f>SUM(D4:D23)</f>
         <v/>
       </c>
-      <c r="E24" s="12" t="n"/>
-      <c r="F24" s="12" t="n"/>
-      <c r="G24" s="12" t="n"/>
-      <c r="H24" s="12" t="n"/>
-      <c r="I24" s="12" t="n"/>
-      <c r="J24" s="12" t="n"/>
-      <c r="K24" s="12" t="n"/>
-      <c r="L24" s="13">
+      <c r="E24" s="11" t="n"/>
+      <c r="F24" s="11" t="n"/>
+      <c r="G24" s="11" t="n"/>
+      <c r="H24" s="11" t="n"/>
+      <c r="I24" s="11" t="n"/>
+      <c r="J24" s="11" t="n"/>
+      <c r="K24" s="11" t="n"/>
+      <c r="L24" s="12">
         <f>SUM(L4:L23)</f>
         <v/>
       </c>
-      <c r="M24" s="12" t="n"/>
-      <c r="N24" s="12" t="n"/>
+      <c r="M24" s="11" t="n"/>
+      <c r="N24" s="11" t="n"/>
     </row>
   </sheetData>
   <autoFilter ref="A3:N24"/>
@@ -9897,21 +9471,21 @@
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="12" t="inlineStr">
+      <c r="A49" s="11" t="inlineStr">
         <is>
           <t>合计</t>
         </is>
       </c>
-      <c r="B49" s="12" t="n"/>
-      <c r="C49" s="12" t="n"/>
-      <c r="D49" s="12" t="n"/>
-      <c r="E49" s="12" t="n"/>
-      <c r="F49" s="12" t="n"/>
-      <c r="G49" s="13">
+      <c r="B49" s="11" t="n"/>
+      <c r="C49" s="11" t="n"/>
+      <c r="D49" s="11" t="n"/>
+      <c r="E49" s="11" t="n"/>
+      <c r="F49" s="11" t="n"/>
+      <c r="G49" s="12">
         <f>SUM(G13:G48)</f>
         <v/>
       </c>
-      <c r="H49" s="13">
+      <c r="H49" s="12">
         <f>SUM(H13:H48)</f>
         <v/>
       </c>

</xml_diff>